<commit_message>
Actualización con nuevos puntajes y mejorea de UI
</commit_message>
<xml_diff>
--- a/SistemaEstrellasAmistad.xlsx
+++ b/SistemaEstrellasAmistad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramir\Documents\cursosProgramacion\CursoHTMLyCSS\ProyectoSistemaDeEstrellasLaAmistad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19A0C368-3FD0-4EAA-8F69-F5963ECA6BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFCA2F93-7034-4882-A241-8EE4FC06B41B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{98485AF0-D9F6-42FB-BB47-AF6B77D1C09B}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="66">
   <si>
     <t>jugador</t>
   </si>
@@ -180,10 +180,52 @@
     <t>Arquero/Medio/Defensa</t>
   </si>
   <si>
-    <t>Director Tecnico</t>
-  </si>
-  <si>
     <t>Agus Distabile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estilo propio </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joaco </t>
+  </si>
+  <si>
+    <t>Enganche / Delantero</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>Gonza Roldan</t>
+  </si>
+  <si>
+    <t>Defensa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sequeira </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Franco </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delantero </t>
+  </si>
+  <si>
+    <t>Chimuelo BOT</t>
+  </si>
+  <si>
+    <t>⭐</t>
+  </si>
+  <si>
+    <t>IA del grupo</t>
+  </si>
+  <si>
+    <t>Director Tecnico(REAL)</t>
+  </si>
+  <si>
+    <t>Norber</t>
+  </si>
+  <si>
+    <t>Lateral derecho</t>
   </si>
 </sst>
 </file>
@@ -550,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A94C24A-CBCB-449A-A6C4-BBCE3B1437D9}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.81640625" customWidth="1"/>
@@ -582,21 +624,21 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -604,10 +646,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
@@ -692,98 +734,98 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B18" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C20" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
         <v>15</v>
@@ -791,10 +833,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
         <v>15</v>
@@ -802,7 +844,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s">
         <v>17</v>
@@ -813,49 +855,134 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C25" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C26" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>58</v>
+      </c>
+      <c r="B29" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>21</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>48</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B35" t="s">
         <v>49</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>50</v>
+      <c r="C35" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C34">
+    <sortCondition descending="1" ref="C2:C34"/>
+  </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>